<commit_message>
feat: add PFC analysis plotting and roadmap update
</commit_message>
<xml_diff>
--- a/Roadmap/Roadmap.xlsx
+++ b/Roadmap/Roadmap.xlsx
@@ -830,12 +830,12 @@
       </c>
       <c r="C17" s="5" t="inlineStr">
         <is>
-          <t>Next</t>
+          <t>Completed</t>
         </is>
       </c>
       <c r="D17" s="2" t="inlineStr">
         <is>
-          <t>Future advanced control capability</t>
+          <t>Implemented PFC foundation: metrics + controller + simulation telemetry + GUI controls/monitoring + dedicated PFC analysis plotting (2026-03-13)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat: add efficiency telemetry and tuning
</commit_message>
<xml_diff>
--- a/Roadmap/Roadmap.xlsx
+++ b/Roadmap/Roadmap.xlsx
@@ -852,12 +852,12 @@
       </c>
       <c r="C18" s="5" t="inlineStr">
         <is>
-          <t>Planned</t>
+          <t>Completed</t>
         </is>
       </c>
       <c r="D18" s="2" t="inlineStr">
         <is>
-          <t>Loss-aware optimization and tradeoff tuning</t>
+          <t>Implemented efficiency telemetry, loss tracking, efficiency analysis plotting, and heuristic tuning recommendations (2026-03-13)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat: extend runtime architecture with startup, inverter realism, hardware backend, and docs
</commit_message>
<xml_diff>
--- a/Roadmap/Roadmap.xlsx
+++ b/Roadmap/Roadmap.xlsx
@@ -2,15 +2,14 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
-  <workbookProtection/>
   <bookViews>
-    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
     <sheet name="Roadmap" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
-  <calcPr calcId="124519" fullCalcOnLoad="1"/>
+  <calcPr calcId="0" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
@@ -26,8 +25,10 @@
       <scheme val="minor"/>
     </font>
     <font>
+      <name val="Calibri"/>
       <b val="1"/>
-      <color rgb="00FFFFFF"/>
+      <color rgb="FFFFFFFF"/>
+      <sz val="11"/>
     </font>
   </fonts>
   <fills count="6">
@@ -39,26 +40,26 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="001F4E78"/>
-        <bgColor rgb="001F4E78"/>
+        <fgColor rgb="FF1F4E78"/>
+        <bgColor rgb="FF1F4E78"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00C6EFCE"/>
-        <bgColor rgb="00C6EFCE"/>
+        <fgColor rgb="FFC6EFCE"/>
+        <bgColor rgb="FFC6EFCE"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00FFEB9C"/>
-        <bgColor rgb="00FFEB9C"/>
+        <fgColor rgb="FFFFEB9C"/>
+        <bgColor rgb="FFFFEB9C"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00D9E1F2"/>
-        <bgColor rgb="00D9E1F2"/>
+        <fgColor rgb="FFD9E1F2"/>
+        <bgColor rgb="FFD9E1F2"/>
       </patternFill>
     </fill>
   </fills>
@@ -93,7 +94,7 @@
     </xf>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
+    <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
   <colors>
@@ -456,8 +457,8 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D19"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <dimension ref="A1:F24"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.88671875" defaultRowHeight="14.4"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
     <col width="66" customWidth="1" min="2" max="2"/>
@@ -817,7 +818,7 @@
         </is>
       </c>
     </row>
-    <row r="17">
+    <row r="17" ht="28.8" customHeight="1">
       <c r="A17" s="2" t="inlineStr">
         <is>
           <t>Phase 3</t>
@@ -839,7 +840,7 @@
         </is>
       </c>
     </row>
-    <row r="18">
+    <row r="18" ht="28.8" customHeight="1">
       <c r="A18" s="2" t="inlineStr">
         <is>
           <t>Phase 3</t>
@@ -861,7 +862,7 @@
         </is>
       </c>
     </row>
-    <row r="19">
+    <row r="19" ht="28.8" customHeight="1">
       <c r="A19" s="2" t="inlineStr">
         <is>
           <t>Phase 4</t>
@@ -874,12 +875,128 @@
       </c>
       <c r="C19" s="5" t="inlineStr">
         <is>
-          <t>Planned</t>
+          <t>In Progress</t>
         </is>
       </c>
       <c r="D19" s="2" t="inlineStr">
         <is>
-          <t>DAQ/real-time target/hardware interface</t>
+          <t>Hardware I/O abstraction layer added to SimulationEngine with mock DAQ backend, runtime enable/disable, diagnostics, and tests (2026-03-15).</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>Phase 3</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>Inverter realism enhancement (switchable multi-physics blocks)</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>Completed</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>Implemented configurable inverter realism: device/dead-time/conduction/switching/diode/min-pulse/bus-ripple/thermal/phase-asymmetry with telemetry, plotting, export, and tests (2026-03-15).</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>Phase 4</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>Hardware integration GUI wiring (mock backend controls)</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>Completed</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>Added GUI controls for enabling mock DAQ backend, noise/seed configuration, engine wiring, export metadata, and regression tests (2026-03-15).</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>Phase 4</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>Hardware monitoring telemetry in GUI</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>Completed</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>Added live monitoring indicators for hardware enabled/connected/backend/write-read counters/I-O error flag in monitoring tab with regression coverage (2026-03-15).</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>Phase 4</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>Communication terminology clarification in GUI</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>Completed</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>Renamed user-facing hardware monitoring/control wording to communication terminology to avoid confusion with inverter hardware modeling (2026-03-15).</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>Phase 4</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>Standard startup sequence (FOC+V/f): align, open-loop ramp, closed-loop handoff</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>Completed</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>Implemented full startup phase machines for FOC and V/f. Sensored FOC skips open-loop phase and goes align-&gt;closed-loop. Added GUI controls, monitoring telemetry, export metadata, and regression tests.</t>
+        </is>
+      </c>
+      <c r="E24" t="inlineStr"/>
+      <c r="F24" t="inlineStr">
+        <is>
+          <t>2026-03-15</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat: unbounded FOC auto-tuning convergence and documentation update (March 2026)
</commit_message>
<xml_diff>
--- a/Roadmap/Roadmap.xlsx
+++ b/Roadmap/Roadmap.xlsx
@@ -457,7 +457,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F24"/>
+  <dimension ref="A1:F25"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.88671875" defaultRowHeight="14.4"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -993,10 +993,36 @@
           <t>Implemented full startup phase machines for FOC and V/f. Sensored FOC skips open-loop phase and goes align-&gt;closed-loop. Added GUI controls, monitoring telemetry, export metadata, and regression tests.</t>
         </is>
       </c>
-      <c r="E24" t="inlineStr"/>
       <c r="F24" t="inlineStr">
         <is>
           <t>2026-03-15</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>Phase 3</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>FOC auto-tuning no-timeout stabilization at 1000 RPM</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>Completed</t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>Adjusted convergence gating: orthogonality check is now load-aware at low Iq, preserving strict gate under meaningful torque; validated accepted/full_converged at 1000 RPM with overcurrent abort policy (2026-03-17).</t>
+        </is>
+      </c>
+      <c r="F25" t="inlineStr">
+        <is>
+          <t>2026-03-17</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Field weakening calibration complete: all 3 motors validated (ME1718, ME1719, Innotec). Multi-motor validation report generated. Efficiency targets met (81.5-83.1%). Documentation updated (ARCHITECTURE.md, Roadmap.md).
</commit_message>
<xml_diff>
--- a/Roadmap/Roadmap.xlsx
+++ b/Roadmap/Roadmap.xlsx
@@ -457,7 +457,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F25"/>
+  <dimension ref="A1:F34"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.88671875" defaultRowHeight="14.4"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -1026,6 +1026,204 @@
         </is>
       </c>
     </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>Phase 4</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>GUI-triggered loaded calibration workflow</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>Planned</t>
+        </is>
+      </c>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>Expose loaded-point calibration directly in the accessible GUI so users can launch it without leaving the application (2026-03-17).</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>Phase 4</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>Single-active-job enforcement for simulation/calibration</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>Planned</t>
+        </is>
+      </c>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>Block new long-running launches while an older simulation or calibration process is still alive; require explicit completion or cancellation first (2026-03-17).</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>Phase 4</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>Process lifecycle tracking and guaranteed shutdown</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>Planned</t>
+        </is>
+      </c>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t>Track every spawned process and ensure it is closed when finished or cancelled, avoiding orphaned workers (2026-03-17).</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>Phase 4</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>Bottom status bar for simulation and process telemetry</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>Planned</t>
+        </is>
+      </c>
+      <c r="D29" t="inlineStr">
+        <is>
+          <t>Add accessible status reporting for active process state, estimated remaining simulation time, and other runtime indicators (2026-03-17).</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>Phase 4</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>PWM-period CPU load estimator</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>Planned</t>
+        </is>
+      </c>
+      <c r="D30" t="inlineStr">
+        <is>
+          <t>Estimate CPU load from control-computation time divided by PWM period budget, matching embedded controller timing analysis (2026-03-17).</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>Phase 5</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>Microcontroller-faithful simulation scheduling</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>Planned</t>
+        </is>
+      </c>
+      <c r="D31" t="inlineStr">
+        <is>
+          <t>Reproduce real MCU sequencing for sampling, control calculation, and command application timing in the simulator (2026-03-17).</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>Phase 5</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>Shunt and differential-amplifier phase-current measurement model</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>Planned</t>
+        </is>
+      </c>
+      <c r="D32" t="inlineStr">
+        <is>
+          <t>Model shunt-based current sensing with amplifier gain, offset, and backward-capacitance-derived cutoff frequency for more realistic hardware behavior (2026-03-17).</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>Phase 5</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>Current-measurement error sensitivity and harmonic impact study</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>Planned</t>
+        </is>
+      </c>
+      <c r="D33" t="inlineStr">
+        <is>
+          <t>Quantify the effect of current-measurement gain and offset errors on control behavior and phase-current harmonics (2026-03-17).</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>Phase 3</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>Voltage-headroom-based field weakening scheduler</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>Completed</t>
+        </is>
+      </c>
+      <c r="D34" t="inlineStr">
+        <is>
+          <t>Reworked FW to regulate dq voltage headroom with tunable target voltage reserve, including GUI wiring and telemetry for injected Id/headroom (2026-03-17).</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
test: extend Phase D GUI integration coverage
- add tests/test_phase_d_gui_extended.py (68 tests)

- update Roadmap/ROADMAP.md with Phase D validation milestones

- record main_window.py coverage increase to 84%
</commit_message>
<xml_diff>
--- a/Roadmap/Roadmap.xlsx
+++ b/Roadmap/Roadmap.xlsx
@@ -457,7 +457,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F34"/>
+  <dimension ref="A1:F35"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.88671875" defaultRowHeight="14.4"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -1224,6 +1224,33 @@
         </is>
       </c>
     </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>Phase 5</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>Topology-aware inverter current-sense GUI and integration validation</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>Completed</t>
+        </is>
+      </c>
+      <c r="D35" t="inlineStr">
+        <is>
+          <t>Added 68 Phase D GUI/integration tests covering lifecycle, calibration completion paths, monitoring updates, FFT window wiring, and current-sense behavior for single/double/triple shunts; main_window.py coverage reached 84% (2026-03-19).</t>
+        </is>
+      </c>
+      <c r="F35" t="inlineStr">
+        <is>
+          <t>2026-03-19</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
feat: complete current-sense measured-vs-true UX and verification
</commit_message>
<xml_diff>
--- a/Roadmap/Roadmap.xlsx
+++ b/Roadmap/Roadmap.xlsx
@@ -457,7 +457,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F35"/>
+  <dimension ref="A1:F36"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.88671875" defaultRowHeight="14.4"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -1251,6 +1251,23 @@
         </is>
       </c>
     </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>2026-03-19</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>Phase D current-sense closure</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>Completed measured-vs-true plot, narrated metrics, integration tests, and validated single-shunt sector-aware behavior</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Release 0.8.0 docs and legal refresh
</commit_message>
<xml_diff>
--- a/Roadmap/Roadmap.xlsx
+++ b/Roadmap/Roadmap.xlsx
@@ -457,7 +457,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F36"/>
+  <dimension ref="A1:F37"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.88671875" defaultRowHeight="14.4"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -1254,17 +1254,54 @@
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
+          <t>Phase 5</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>Phase D current-sense closure</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>Completed</t>
+        </is>
+      </c>
+      <c r="D36" t="inlineStr">
+        <is>
+          <t>Completed measured-vs-true current history, reconstructed-current FOC feedback, single-shunt physical bridge correction, FFT units/exports, and narrated analysis workflow (2026-03-19).</t>
+        </is>
+      </c>
+      <c r="F36" t="inlineStr">
+        <is>
           <t>2026-03-19</t>
         </is>
       </c>
-      <c r="B36" t="inlineStr">
-        <is>
-          <t>Phase D current-sense closure</t>
-        </is>
-      </c>
-      <c r="C36" t="inlineStr">
-        <is>
-          <t>Completed measured-vs-true plot, narrated metrics, integration tests, and validated single-shunt sector-aware behavior</t>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>Phase 5</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>Release 0.8.0 documentation and legal refresh</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>Completed</t>
+        </is>
+      </c>
+      <c r="D37" t="inlineStr">
+        <is>
+          <t>Normalized project version to 0.8.0, added license/disclaimer headers across docs, updated Sphinx/README/release notes for current-sense and FFT features, and regenerated HTML docs (2026-03-19).</t>
+        </is>
+      </c>
+      <c r="F37" t="inlineStr">
+        <is>
+          <t>2026-03-19</t>
         </is>
       </c>
     </row>

</xml_diff>